<commit_message>
Update bug reports and Test case in Search module
</commit_message>
<xml_diff>
--- a/Manual Test _ Instagram.xlsx
+++ b/Manual Test _ Instagram.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LOQ\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F40EE96B-0FDD-449E-B685-5531C5924AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE33A13-87D5-4D9E-BAA5-C394BB9D593A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="3" xr2:uid="{6A5DBA80-7A46-4704-8A6F-7ED5D94F7523}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{6A5DBA80-7A46-4704-8A6F-7ED5D94F7523}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="170">
   <si>
     <t>ID</t>
   </si>
@@ -540,9 +540,6 @@
     <t>Open</t>
   </si>
   <si>
-    <t>Attatchment</t>
-  </si>
-  <si>
     <t>Login successfully with phone number</t>
   </si>
   <si>
@@ -555,12 +552,6 @@
 4. Click button Login - or press Enter</t>
   </si>
   <si>
-    <t>Return to Search page from the Profile page of an account</t>
-  </si>
-  <si>
-    <t>From profile page, redirecting back to Search page with the current search context and results list</t>
-  </si>
-  <si>
     <t>There is no such button to go back to search page.</t>
   </si>
   <si>
@@ -568,25 +559,6 @@
   </si>
   <si>
     <t>Test case ID</t>
-  </si>
-  <si>
-    <t>1. Access instagram Feed page: https://www.instagram.com/explore/
-2. Click on the Search input
-3. Enter username/display of an existent account
-4. Choose one to redirect to the account profile page
-5. Click "&lt;" button to go back to Search page</t>
-  </si>
-  <si>
-    <t>1. Access instagram Feed page: https://www.instagram.com/explore/
-2. Click on the Search input
-3. Enter username/display of an existent account
-4. Choose one to redirect to the account profile page</t>
-  </si>
-  <si>
-    <t>The backward button with "&lt;" icon is at the top left corner next to account information display section. Click to go back to Search page with current search context and results list</t>
-  </si>
-  <si>
-    <t>No backward button available on the chosen account profile page</t>
   </si>
   <si>
     <t>1. Access instagram Feed page: https://www.instagram.com/
@@ -611,19 +583,49 @@
     <t>Image and video</t>
   </si>
   <si>
-    <t>Preconditon</t>
-  </si>
-  <si>
-    <t>Browser is full screen</t>
-  </si>
-  <si>
     <t>Video</t>
   </si>
   <si>
-    <t>[Functional] There is no backward button to go back to Search page from an account Profile page</t>
-  </si>
-  <si>
-    <t>[UI] Search field overflows and search results list is overlapped by Reels section on smaller screen</t>
+    <t>[Search] No "Back" button displayed on the user Profile page to return to the Search results</t>
+  </si>
+  <si>
+    <t>1. User is logged in to Instagram.
+2. Browser window is maximized (Full screen).</t>
+  </si>
+  <si>
+    <t>User is logged in to Instagram.</t>
+  </si>
+  <si>
+    <t>1. Access instagram Explore page: https://www.instagram.com/explore/
+2. Click on the Search bar
+3. Enter username/display of an existing account
+4. Click on the user account from the dropdown list</t>
+  </si>
+  <si>
+    <t>There is no "Back" button available on the visited profile page.</t>
+  </si>
+  <si>
+    <t>A "Back" button (with "&lt;" icon) should be displayed at the top-left corner next to the account name.
+Clicking this button should return the user to the Search page while retaining the current search context and results.</t>
+  </si>
+  <si>
+    <t>Attachment</t>
+  </si>
+  <si>
+    <t>[Search] Search field overflows and search results list is overlapped by Reels section on smaller screen</t>
+  </si>
+  <si>
+    <t>Return to Search page from the visited profile page of an account</t>
+  </si>
+  <si>
+    <t>1. Access instagram Feed page: https://www.instagram.com/explore/
+2. Click on the Search bar
+3. Enter username/display of an existent account
+4. Click on the user account from the dropdown list
+5. Click "&lt;" button to go back to Search page</t>
+  </si>
+  <si>
+    <t>From profile page, redirecting back to Search page while retaining the current search context and results.</t>
   </si>
 </sst>
 </file>
@@ -718,16 +720,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1530,32 +1529,32 @@
         <v>111</v>
       </c>
     </row>
-    <row r="22" spans="8:16" s="8" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="H22" s="6" t="s">
+    <row r="22" spans="8:16" s="7" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="H22" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I22" s="6" t="s">
+      <c r="I22" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="J22" s="7" t="s">
+      <c r="J22" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="K22" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="K22" s="1" t="s">
+      <c r="L22" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="L22" s="1" t="s">
-        <v>150</v>
       </c>
       <c r="M22" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="N22" s="6" t="s">
+      <c r="N22" s="5" t="s">
         <v>40</v>
       </c>
       <c r="O22" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P22" s="6" t="s">
+      <c r="P22" s="5" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1843,33 +1842,33 @@
         <v>111</v>
       </c>
     </row>
-    <row r="19" spans="8:16" s="8" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="H19" s="6" t="s">
+    <row r="19" spans="8:16" s="7" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="H19" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="I19" s="6" t="s">
+      <c r="I19" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="J19" s="7" t="s">
+      <c r="J19" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="M19" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="N19" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="O19" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="P19" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="K19" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="L19" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="M19" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="N19" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="O19" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="P19" s="6" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="20" spans="8:16" ht="57.6" x14ac:dyDescent="0.3">
@@ -2229,7 +2228,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E32E2B9-6C69-4EE3-8F2B-3682AD23456D}">
-  <dimension ref="D4:E33"/>
+  <dimension ref="D4:E32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="17.21875" style="1" bestFit="1" customWidth="1"/>
@@ -2237,213 +2236,205 @@
   </cols>
   <sheetData>
     <row r="4" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="5" spans="4:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="6" spans="4:5" s="3" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D6" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>56</v>
+      <c r="E5" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D6" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="4:5" ht="26.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D8" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="9" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D9" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="10" spans="4:5" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D10" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="11" spans="4:5" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D11" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="12" spans="4:5" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D12" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="13" spans="4:5" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D13" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="14" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="15" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D15" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E15" s="3"/>
+    </row>
+    <row r="20" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D20" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="21" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D21" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="4:5" ht="37.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D22" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="23" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D23" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="8" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D8" s="5" t="s">
+      <c r="E23" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="4:5" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D9" s="5" t="s">
+      <c r="E24" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="4:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D25" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="26" spans="4:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D26" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="27" spans="4:5" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D27" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="10" spans="4:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D10" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="11" spans="4:5" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D11" s="5" t="s">
+      <c r="E27" s="8" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="28" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D28" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="12" spans="4:5" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D12" s="5" t="s">
+      <c r="E28" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="29" spans="4:5" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D29" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="13" spans="4:5" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D13" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="E13" s="10" t="s">
+      <c r="E29" s="3" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="14" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D14" s="5" t="s">
+    <row r="30" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D30" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="31" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D31" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E31" s="3" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="15" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D15" s="5" t="s">
+    <row r="32" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D32" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E15" s="4"/>
-    </row>
-    <row r="20" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D20" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="21" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D21" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="22" spans="4:5" ht="37.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D22" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="23" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D23" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="24" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D24" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="25" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D25" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D26" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="27" spans="4:5" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D27" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="28" spans="4:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D28" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="29" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D29" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="30" spans="4:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D30" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="31" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D31" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="32" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D32" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="33" spans="4:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D33" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="E33" s="4"/>
+      <c r="E32" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E13" r:id="rId1" xr:uid="{5D000EAF-9A33-4EFE-B37B-EB902B2BAE8D}"/>
-    <hyperlink ref="E31" r:id="rId2" xr:uid="{00708FFC-155B-446D-939F-7A5086202B07}"/>
+    <hyperlink ref="E30" r:id="rId2" xr:uid="{00708FFC-155B-446D-939F-7A5086202B07}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>